<commit_message>
adapters: ship GENERIC renderers with the adapter (docx/xlsx); drop instance scripts
Renderers must be universal/instance-agnostic (no product data) so they travel with
the framework and keep the base neutral. to-document/render.py (markdown -> styled
.docx) and to-table/render.py (markdown tables from any instance -> .xlsx/CSV) now live
in the adapter folders; the decksmith-specific renderers/ folder is removed. Adapters
stay instruction-skills by default; a render.py ships ONLY where a library is required.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/decksmith/deliverables/decksmith-registers-and-plan.xlsx
+++ b/examples/decksmith/deliverables/decksmith-registers-and-plan.xlsx
@@ -99,9 +99,7 @@
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -482,22 +480,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="46" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="54" customWidth="1" min="6" max="6"/>
+    <col width="54" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Hypotheses — source: registers/hypotheses.md · rendered 2026-07-21 (to-table)</t>
+          <t>source: registers/hypotheses.md · rendered 2026-07-21 (to-table)</t>
         </is>
       </c>
     </row>
@@ -529,10 +528,15 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
           <t>Test</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
@@ -546,7 +550,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Engine reliably produces native files both genuinely editable AND well-designed, at scale</t>
+          <t>The engine can reliably produce native files that are both genuinely editable and genuinely well-designed, at scale</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -566,12 +570,17 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Step4 M-edit-fidelity &gt;=90% (fail &lt;70%); Step5 20 test decks + rule; Step6 F-1+T-1 first read</t>
+          <t>concept (../passport.md#concept)</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>assumption</t>
+          <t>Step 4: M-edit-fidelity ≥ 90% (fail &lt; 70%) · Step 5: 20 test decks, decision rule set (../tactical-plan.md#hypotheses-to-test) · Step 6: F-1+T-1 produce first read (../sprint-plan.md#must)</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>[assumption]</t>
         </is>
       </c>
     </row>
@@ -583,7 +592,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Salespeople &amp; marketers are a reachable segment who feel 'AI decks look templated' (P1) enough to switch</t>
+          <t>Salespeople &amp; marketers are a reachable segment who feel "AI decks look templated" (P1) strongly enough to switch</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -603,12 +612,17 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>discovery interviews + demand test (Step 5)</t>
+          <t>segments/problems (../passport.md#problems)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>assumption</t>
+          <t>discovery interviews + a demand test (Step 5)</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>[assumption]</t>
         </is>
       </c>
     </row>
@@ -620,7 +634,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>'Wrong structure/framing' (P2) is a top pain worth solving, not just styling slides</t>
+          <t>"Wrong structure/framing" (P2) is a top pain worth solving, not just styling slides</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -640,12 +654,17 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
+          <t>problems (../passport.md#problems)</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
           <t>discovery interviews (Step 5)</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>assumption</t>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>[assumption]</t>
         </is>
       </c>
     </row>
@@ -657,7 +676,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>The editable-and-beautiful quality is defensible (survives an LLM rebuild); pressured at Step 2 by Copilot/Canva</t>
+          <t>The engine's editable-and-beautiful quality is defensible — hard to replicate cheaply, survives an LLM rebuild. Pressured at Step 2: incumbents (Copilot/Canva) are entering the wedge, so the moat must be the fidelity+design *engine*, not the app</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -677,12 +696,17 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
+          <t>value (../passport.md#value-defensibility); pressured by ../analysis.md#competitor-strategy</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
           <t>observe replication attempts / sustained quality gap (Step 3+)</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>assumption</t>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>[assumption]</t>
         </is>
       </c>
     </row>
@@ -694,7 +718,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>A native high-fidelity editable+designed deck is a real unmet need valued over web-format generation</t>
+          <t>A native, high-fidelity editable-and-designed deck is a real unmet need the lead segment values over web-format generation (Gamma's .pptx export flattens 30–40% of slides)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -714,12 +738,17 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Step4 M-activation &gt;=30% (fail &lt;10%); Step5 demand probe B-01/B-03 &gt;=10 trials; Step6 A-1 seeds B-01</t>
+          <t>opportunity/substitutes (../analysis.md#opportunity)</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>assumption</t>
+          <t>Step 4: M-activation ≥ 30% (fail &lt; 10%) · Step 5: demand probe B-01/B-03, ≥ 10 qualified trials (../tactical-plan.md#hypotheses-to-test) · Step 6: A-1 seeds B-01 probe (../sprint-plan.md#must)</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>[assumption]</t>
         </is>
       </c>
     </row>
@@ -731,7 +760,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>The obtainable market is large enough to build a business on (bottom-up SAM ~$750M)</t>
+          <t>The obtainable market is large enough to build a business on (bottom-up SAM ~$750M; realistic SOM)</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -751,12 +780,17 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>validate reachable-count + price + adoption (Step 4)</t>
+          <t>market-sizing (../analysis.md#market-sizing)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>assumption</t>
+          <t>validate reachable-count + price + adoption assumptions (Step 4)</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>[assumption]</t>
         </is>
       </c>
     </row>
@@ -768,7 +802,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>For the beachhead job, actually-editable + designed native decks is a strong enough wedge to switch</t>
+          <t>For the beachhead job, "actually-editable + designed native decks" is a strong enough wedge that salespeople &amp; marketers switch (pull beats the "I'll still have to fix it" anxiety + PowerPoint habit)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -788,12 +822,17 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Step4 M-wk-retention flattens &gt;0; demand test (Step 5)</t>
+          <t>bets (../strategy.md#bets); job/forces (../passport.md#jtbd)</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>assumption</t>
+          <t>Step 4: M-wk-retention flattens &gt; 0; demand test (Step 5)</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>[assumption]</t>
         </is>
       </c>
     </row>
@@ -805,7 +844,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>A standalone native-fidelity+design engine can stay ahead of incumbents long enough to build lock-in</t>
+          <t>A standalone native-fidelity+design engine can stay ahead of incumbents (Copilot/Canva) closing the wedge long enough to build lock-in</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -825,12 +864,17 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
+          <t>bets (../strategy.md#bets); ../analysis.md#opportunity</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
           <t>sustained quality gap + retention once customers exist (pmf)</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>assumption</t>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>[assumption]</t>
         </is>
       </c>
     </row>
@@ -842,7 +886,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>The beachhead will pay a standalone subscription (~$15-25) despite incumbents bundling</t>
+          <t>The beachhead will pay a standalone subscription (~$15–25) despite incumbents bundling</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -862,12 +906,17 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Step4 WTP &gt;=$15/mo (fail &lt;$10); price-talk pilot (Step 5)</t>
+          <t>pricing (../strategy.md#pricing)</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>assumption</t>
+          <t>Step 4: WTP ≥ $15/mo (fail &lt; $10); price-talk pilot (Step 5)</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>[assumption]</t>
         </is>
       </c>
     </row>
@@ -899,18 +948,23 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
+          <t>channels (../strategy.md#channels-expansion)</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
           <t>channel tests with pre-set CAC threshold (Step 5)</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>assumption</t>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>[assumption]</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -926,20 +980,20 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="46" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="54" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Risks — source: registers/risks.md · rendered 2026-07-21 (to-table)</t>
+          <t>source: registers/risks.md · rendered 2026-07-21 (to-table)</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1077,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>founder</t>
+          <t>⚙️ founder</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -1033,7 +1087,7 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>Step 2</t>
+          <t>Step 2 (../analysis.md#niche-risks)</t>
         </is>
       </c>
     </row>
@@ -1045,7 +1099,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Incumbents (Copilot in PPT, Canva AI) bundle native-editable AI generation with distribution</t>
+          <t>Incumbents (Microsoft Copilot in PPT, Canva AI 2.0) bundle native-editable AI generation with distribution — closes our wedge</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -1065,12 +1119,12 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>Move fast on the fidelity gap; position sharply on 'actually editable'; track releases</t>
+          <t>Move fast on the fidelity gap; position sharply on "actually editable"; track their releases</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>founder / ongoing</t>
+          <t>⚙️ founder · ongoing</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
@@ -1080,7 +1134,7 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>Step 2</t>
+          <t>Step 2 (../analysis.md#substitutes)</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1146,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Capable buyers self-build with general LLMs (ChatGPT/Claude) — caps willingness to pay</t>
+          <t>Capable buyers self-build with general LLMs (ChatGPT/Claude) → caps willingness to pay for "just generate slides"</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1117,7 +1171,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>founder</t>
+          <t>⚙️ founder</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -1127,7 +1181,7 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Step 2</t>
+          <t>Step 2 (../analysis.md#substitutes)</t>
         </is>
       </c>
     </row>
@@ -1159,12 +1213,12 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Abstract the provider (multi-model); cap M-cogs-per-deck; keep the engine in-house</t>
+          <t>Abstract the provider (multi-model); cap M-cogs-per-deck; keep the fidelity engine in-house</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>eng / ongoing</t>
+          <t>⚙️ eng · ongoing</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -1174,7 +1228,7 @@
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>Step 2</t>
+          <t>Step 2 (../analysis.md#niche-risks)</t>
         </is>
       </c>
     </row>
@@ -1186,7 +1240,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Low entry barrier for 'AI slide wrappers' — crowded, fast-moving rivalry</t>
+          <t>Low entry barrier for "AI slide wrappers" → crowded, fast-moving rivalry</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1211,7 +1265,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>founder</t>
+          <t>⚙️ founder</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -1221,7 +1275,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Step 2</t>
+          <t>Step 2 (../analysis.md#niche-risks)</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1312,7 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>founder</t>
+          <t>⚙️ founder</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -1268,7 +1322,7 @@
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>Step 2</t>
+          <t>Step 2 (../analysis.md#substitutes)</t>
         </is>
       </c>
     </row>
@@ -1280,7 +1334,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>The engine never reliably hits native-fidelity + design at scale — whole strategy rests on H-001</t>
+          <t>The engine never reliably hits native-fidelity + design at scale — the whole strategy rests on one feasibility bet (H-001)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1300,12 +1354,12 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Build a thin vertical slice first; gate on M-edit-fidelity &gt;=90% before investing further</t>
+          <t>Build the fidelity engine as a thin vertical slice first; gate on M-edit-fidelity ≥ 90% before investing further</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>founder/eng / next sprint</t>
+          <t>⚙️ founder/eng · next sprint</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1315,7 +1369,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Step 3</t>
+          <t>Step 3 (../strategy.md#product-risks)</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1381,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>The beachhead won't pay standalone vs bundled incumbents ($15-30 bundled) — no viable revenue</t>
+          <t>The beachhead won't pay standalone vs bundled incumbents (Copilot/Canva at $15–30 bundled) → no viable revenue</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -1347,12 +1401,12 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>Test WTP early (Step 5 pilot) before building billing; don't scale spend until validated</t>
+          <t>Test WTP early (Step 5 pilot) before building billing; don't scale spend until the wedge is validated</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>founder / Step 5</t>
+          <t>⚙️ founder · Step 5</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -1362,7 +1416,7 @@
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>Step 3</t>
+          <t>Step 3 (../strategy.md#pricing)</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1428,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Community + product-led virality doesn't materialize — CAC too high to grow</t>
+          <t>Community + product-led virality doesn't materialize → CAC too high to grow</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1399,7 +1453,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>founder / Step 5</t>
+          <t>⚙️ founder · Step 5</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1409,7 +1463,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Step 3</t>
+          <t>Step 3 (../strategy.md#channels-expansion)</t>
         </is>
       </c>
     </row>
@@ -1432,18 +1486,18 @@
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="54" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="33" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Metric tree (definitions) — source: registers/metric-tree.md · rendered 2026-07-21 (to-table) · concept stage: all not-instrumented, no readings</t>
+          <t>source: registers/metric-tree.md · rendered 2026-07-21 (to-table)</t>
         </is>
       </c>
     </row>
@@ -1497,7 +1551,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>North Star (candidate). Decks generated -&gt; exported -&gt; kept and edited per active deck-maker per week. A redo = value failed, so it encodes 'editable AND designed'.</t>
+          <t>North Star (⚙️ candidate). Decks generated → exported → kept and edited (used as the real deliverable, not rebuilt by hand) per active deck-maker per week. A redo = the value failed, so this encodes "editable and designed".</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -1522,7 +1576,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>grow</t>
+          <t>⚙️ grow</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -1539,7 +1593,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>THE concept-proving metric. Share of exported slide objects that are natively editable (real shapes/text, not flattened images) — the anti-Gamma metric.</t>
+          <t>THE concept-proving metric. Share of exported slide objects that are natively editable (real shapes/text, not flattened images) — the anti-Gamma metric; proxy for "I don't have to redo it".</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -1564,7 +1618,7 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>&gt;= 90%</t>
+          <t>⚙️ ≥ 90%</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
@@ -1581,7 +1635,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Share of new signups who generate AND export a first editable deck &lt;= 7d.</t>
+          <t>Share of new signups who generate AND export a first editable deck ≤ 7d.</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1606,7 +1660,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>to clarify</t>
+          <t>— to clarify —</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -1648,7 +1702,7 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>to clarify (no cohorts)</t>
+          <t>— to clarify — (no cohorts yet)</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -1665,7 +1719,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Free -&gt; paid conversion &lt;= 30d (full funnel).</t>
+          <t>Free → paid conversion ≤ 30d (full funnel).</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1690,7 +1744,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>to clarify</t>
+          <t>— to clarify —</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -1707,7 +1761,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>LLM inference + render cost per generated deck (COGS).</t>
+          <t>LLM inference + render cost per generated deck (COGS). basis: metered = API list price; fact = real spend.</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -1732,7 +1786,7 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>down</t>
+          <t>⚙️ ↓</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -1749,7 +1803,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>(Revenue - COGS) / Revenue.</t>
+          <t>(Revenue − COGS) / Revenue.</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1774,7 +1828,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>&gt;= 70%</t>
+          <t>⚙️ ≥ 70%</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1801,24 +1855,24 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="54" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Strategic plan — global hypotheses (quantified bets) — source: strategic-plan.md#global-hypotheses · rendered 2026-07-21 (to-table)</t>
+          <t>source: strategic-plan.md#global-hypotheses · rendered 2026-07-21 (to-table)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>H-…</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1828,7 +1882,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Metric node</t>
+          <t>Metric node (M-…)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1865,7 +1919,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>&gt;= 90% objects natively editable</t>
+          <t>⚙️ ≥ 90% objects natively editable</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -1875,7 +1929,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>assumption</t>
+          <t>[assumption]</t>
         </is>
       </c>
     </row>
@@ -1897,7 +1951,7 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>&gt;= 30% activate (generate+export+keep)</t>
+          <t>⚙️ ≥ 30% activate (generate+export+keep)</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -1907,7 +1961,7 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>assumption</t>
+          <t>[assumption]</t>
         </is>
       </c>
     </row>
@@ -1929,7 +1983,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>retention curve flattens &gt; 0</t>
+          <t>⚙️ retention curve flattens &gt; 0</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -1939,7 +1993,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>assumption</t>
+          <t>[assumption]</t>
         </is>
       </c>
     </row>
@@ -1956,12 +2010,12 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>WTP -&gt; M-free-paid-conv</t>
+          <t>(WTP → M-free-paid-conv)</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>WTP &gt;= $15/mo in pilot</t>
+          <t>⚙️ WTP ≥ $15/mo in pilot</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -1971,7 +2025,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>assumption</t>
+          <t>[assumption]</t>
         </is>
       </c>
     </row>
@@ -1989,63 +2043,57 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="54" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Sprint 1 plan (must + backlog) — source: sprint-plan.md#must / #backlog · rendered 2026-07-21 (to-table)</t>
+          <t>source: sprint-plan.md#backlog · rendered 2026-07-21 (to-table)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tier</t>
+          <t>Rank</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Rank</t>
+          <t>Direction</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Direction</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Format</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Format</t>
+          <t>Links (H-…/M-…)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Links</t>
+          <t>Est.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Est.</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
@@ -2054,318 +2102,191 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>must</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>back-office</t>
+        </is>
+      </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>development</t>
+          <t>T-2 · Assemble the 20 representative test decks (layouts, charts, images that fairly stress fidelity) — DoD: 20 decks agreed as representative, versioned</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>F-1 Native .pptx export slice (generate -&gt; export one deck)</t>
+          <t>Task+DoD</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>M-edit-fidelity · R-007</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>H-001 / M-edit-fidelity</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>assumption</t>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>[assumption]</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>must</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>back-office</t>
+        </is>
+      </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>go-to-market</t>
+          <t>T-3 · Abstract the LLM provider behind one interface (swap without rewrite) — DoD: provider swappable via config; one alt tested</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>A-1 Seed the demand probe in one sales-enablement community (B-01)</t>
+          <t>Task+DoD</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>M-cogs-per-deck · R-004</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>H-005 / M-activation</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>assumption</t>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>[assumption]</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>must</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>go-to-market</t>
+        </is>
+      </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>back-office</t>
+          <t>A-2 · Intent SEO page "fix Gamma PPT export" (B-03) — capture the Gamma-frustrated intent, route to trial</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>T-1 Edit-fidelity measurement harness + export event capture</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Task+DoD</t>
+          <t>H-005 / M-activation</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>M-edit-fidelity / M-activation / R-007</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>assumption</t>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>[assumption]</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>backlog</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>development</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>back-office</t>
+          <t>F-2 · Brand-kit intake (upload colors/fonts → applied to export) for the marketer bundle B-02</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>T-2 Assemble the 20 representative test decks</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Task+DoD</t>
+          <t>H-007 / M-activation</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>M-edit-fidelity / R-007</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>assumption</t>
+          <t>[assumption]</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>backlog</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>development</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>back-office</t>
+          <t>F-3 · Chart-fidelity hardening (native editable charts beyond the one type in F-1)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>T-3 Abstract the LLM provider behind one interface</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Task+DoD</t>
+          <t>H-001 / M-edit-fidelity</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>M-cogs-per-deck / R-004</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>assumption</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>backlog</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>go-to-market</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>A-2 Intent SEO page 'fix Gamma PPT export' (B-03)</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>H-005 / M-activation</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>assumption</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>backlog</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>development</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>F-2 Brand-kit intake (B-02)</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>H-007 / M-activation</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>assumption</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>backlog</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>development</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>F-3 Chart-fidelity hardening</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>H-001 / M-edit-fidelity</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>assumption</t>
+          <t>[assumption]</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>